<commit_message>
fixes de orden de la GI
</commit_message>
<xml_diff>
--- a/StructureDefinition-convergence-assessment.xlsx
+++ b/StructureDefinition-convergence-assessment.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-11T00:16:12+00:00</t>
+    <t>2026-10-19T22:17:00-03:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1758,17 +1758,17 @@
   <dimension ref="A1:AP51"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="38.30078125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="38.30078125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="39.10546875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="39.10546875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="9.984375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="34.8125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.29296875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.21484375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.55078125" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.1171875" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="10.75390625" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="122.43359375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="129.546875" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1777,28 +1777,28 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.53515625" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="54.6171875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="47.7421875" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="35.16796875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="7.93359375" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="14.08984375" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="14.4296875" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="15.31640625" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="14.62890625" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="54.2734375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="50.55078125" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.10546875" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="17.6953125" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="15.98046875" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="13.44140625" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="11.03515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="36.046875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="8.51953125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="8.859375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="25.4609375" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="212.10546875" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="23.9609375" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="214.97265625" customWidth="true" bestFit="true"/>
     <col min="39" max="39" width="255.0" customWidth="true" bestFit="true"/>
-    <col min="40" max="40" width="91.75" customWidth="true" bestFit="true"/>
-    <col min="41" max="41" width="31.65234375" customWidth="true" bestFit="true"/>
-    <col min="42" max="42" width="36.3046875" customWidth="true" bestFit="true"/>
+    <col min="40" max="40" width="93.1640625" customWidth="true" bestFit="true"/>
+    <col min="41" max="41" width="29.45703125" customWidth="true" bestFit="true"/>
+    <col min="42" max="42" width="33.8203125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>